<commit_message>
Se incluye links de Falabella y Laskin
</commit_message>
<xml_diff>
--- a/data/productos.xlsx
+++ b/data/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WCORREA\Documents\ISDIN_Shopping_de_precios\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE794A12-FC4F-4385-BEE0-ABACC37DEE54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E20F8B97-F0C9-4DC9-90C2-06F796E141A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{60233B49-B589-B346-B71C-4D486694C55A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$514</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$581</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2056" uniqueCount="633">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2872" uniqueCount="839">
   <si>
     <t>Producto</t>
   </si>
@@ -1938,6 +1938,624 @@
   </si>
   <si>
     <t>https://www.cutis.com.co/isdinceutics-salicylic-renewal-30ml/p</t>
+  </si>
+  <si>
+    <t>Laskin</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/eryfotona-ak-nmsc-spf-99-50ml-flid-isdi?srsltid=AfmBOoqajYIr4FULRRthYuW3-KmIpF-hDl6H6O8RFy5zTySRgE9hLArP</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/essential-cleansing-200ml-oil-base-clean?_pos=1&amp;_sid=520745000&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-fotoprotector-pediatrics-gel-cream-isdin%C2%AE?_pos=2&amp;_sid=e94934467&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprot-invisible-stick-spf50-10g-isdin?_pos=1&amp;_sid=c2b7bf035&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprot-fusion-water-magic-by-alcaraz?srsltid=AfmBOopqsE8lIBNgc4E1YJQcy5uSJdX7fUy9ph9lqks6Q_F1pLmG-LdD</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotec-fusion-gel-sport-spf-50-100ml?_pos=1&amp;_sid=37f59b04f&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotop-fusion-water-col-light-spf50-50ml?_pos=1&amp;_sid=0b71c0477&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotop-fusion-water-col-medium-spf50-50ml?_pos=2&amp;_sid=0b71c0477&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fusion-water-magic-spf-50-isdin%C2%AE?_pos=1&amp;_sid=3207ee7d2&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotec-pediatrics-fision-water-50ml?srsltid=AfmBOoqq5j59XYzMFA4VyDGM7JhXPUSsbojYQgxw5oDJVhqCG102ptfw</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotector-spf-50-250ml-gel-crema?_pos=1&amp;_sid=4e2804c3b&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/foto-ultra-100-50ml-active-unify-ff?_pos=2&amp;_sid=62a048b95&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/foto-ultra-100-50ml-active-unify-color?_pos=1&amp;_sid=62a048b95&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-fotoprotector-magic-repair-50ml</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/reparador-labial-fluid-10-ml-isdin?_pos=1&amp;_sid=1da354c34&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/a-g-e-reverse-day-50ml-cream-isdinceuti?srsltid=AfmBOoqMVJvHzOLWvGqWHaAIZ3w_ivWSYbaV24CoBuJAedpKRuBqw6jj</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/a-g-e-age-reverse-night-50ml-crema-repar?_pos=1&amp;_sid=a24239ed5&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/flavo-c-30ml-serum-isdinceutics?_pos=1&amp;_sid=2a9d540fb&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/hyaluronic-concentrate-30ml-serum-isdinc?_pos=1&amp;_sid=7c34e631e&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/hyaluronic-moisture-normal-cream-50g-isd?_pos=1&amp;_sid=6f9c48e6c&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/k-ox-eyes-15gr-cream-isdinceutics?_pos=2&amp;_sid=80c075cb9&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/melaclear-advanced-serum-30ml-isdinceut?_pos=1&amp;_sid=1deb452d2&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/vital-eyes-15gr-crema-isdinceutics?_pos=1&amp;_sid=34fa6f106&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/retinal-intense-50ml-serum-isdinceutics?_pos=1&amp;_sid=c083a09f4&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-fotoprotector-pediatrics-stick-20g?srsltid=AfmBOopkdGtyZSzBBb4fhL-ujgjUKvcM_z_O1P9vAdCC6QeU4NehDFZ1</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotect-uv-mineral-brush-spf-50-2gr?_pos=1&amp;_sid=ff2decddf&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotector-compact-light-spf-50-10gr?srsltid=AfmBOoozsBArCJGklZqa3JjOV5j_okaT2Pd_44UngFzBuvvTzOMMtBkp</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotector-fusion-fluid-mineral-spf50?_pos=5&amp;_sid=3ce86d8ab&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotop-fusion-water-col-bronz-spf50-50ml?_pos=3&amp;_sid=b5ba19b41&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprot-fusion-water-urban-spf-30-50ml?_pos=2&amp;_sid=30da8fe70&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprotector-fusion-water-magic-gl-50ml?_pos=1&amp;_sid=53a36d7c4&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoprot-transparent-spf-50-250ml-spray?srsltid=AfmBOorqPQXV8gEhZSigizJZjpgmvaqDYGXlPFOHk8CUk83zVROCSD_z</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoultra-redness-spf50-x-50ml-isdin?_pos=1&amp;_sid=fdc18e217&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/foto-ultra-100-50ml-spot-prevent-spf-51?_pos=1&amp;_sid=b02e06879&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/fotoultra-100-spot-prevent-color-spf50?_pos=2&amp;_sid=d3d08e4c5&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-fotoprotec-magic-repair-color-50ml?srsltid=AfmBOooc2NsVaMWEeqekNkNRNdUiEVWoH-A9Es6_oR4CAYKdaQkwYdhT</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ultra-suave-daylisdin-400ml-shampoo?_pos=1&amp;_sid=444677080&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/germisdin-500ml-gel-de-bano-syndet?_pos=1&amp;_sid=c051e5e73&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/anticaida-lambdapil-shampoo-200ml?_pos=1&amp;_sid=94972668f&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/nutradeica-ds-50ml-gel-crema-facial?_pos=1&amp;_sid=97248bac2&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/anticaspa-grasa-nutradeica-200ml-shampo?_pos=1&amp;_sid=a3461daa4&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isd-crema-emol-pro-amp-nutratopic-50ml?_pos=1&amp;_sid=6edad3634&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/nutratopic-pro-amp-400ml-gel-de-bano-emu?_pos=1&amp;_sid=9a8505bb4&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/nutratopic-pro-amp-400ml-locion-emolient?_pos=1&amp;_psq=NUTRATOPIC+LOTION+400ML&amp;_ss=e&amp;_v=1.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/baby-naturals-nutraisdin-pomada-de-panal?srsltid=AfmBOoq-LgO2bhHaMBsEnEwtJemaj7DOIo9wx9gn0oKJ7iEgQw0DYrar</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/baby-naturals-nutraisdin-gel-champu-400m?_pos=1&amp;_sid=afaa20697&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/reparador-labial-stick-rojo-4g?_pos=1&amp;_sid=dfdfa9bd2&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/reparador-labial-stick-rosa?_pos=2&amp;_sid=6f945075d&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/reparador-labial-stick-granate-4g?_pos=1&amp;_sid=0ff523dbc&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/reparador-labial-acido-hialuronico-4gr?_pos=1&amp;_sid=4fe719064&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/si-nails-2-5ml-fortalecedor-de-unas?_pos=1&amp;_sid=d8d752101&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/niogermox-3-3ml-solucion-topica-una?_pos=1&amp;_sid=a8a322ba5&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/micellar-solution-4-en-1-400ml-isdin?_pos=1&amp;_sid=613657c30&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-bath-gel-hydrating-400ml-isdin?_pos=1&amp;_sid=07b0ba64e&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-podos-75ml-gel-oil-hidrat-isd?_pos=1&amp;_sid=ea576f988&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-ultra-10-400ml-locion-plus-repar?_pos=1&amp;_sid=ae74f5a8c&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-lotion-10-hidrat-isdin-1000ml?_pos=1&amp;_sid=834e38f88&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-ultra-20-100ml-crema-anti-rugosi?_pos=1&amp;_sid=f5978cf5e&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/ureadin-manos-plus-50ml-crema-repair?_pos=1&amp;_sid=093618c0b&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/woman-reafirmante-firming-200ml?_pos=1&amp;_sid=281775c23&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdinceutics-hyaluronic-eyes-15g?_pos=1&amp;_sid=1b300de73&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/hyaluronic-moisture-oily-y-cobination-cr?_pos=1&amp;_sid=133e64fc6&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdinceutics-hyaluronic-booster-x-10-amp?_pos=1&amp;_sid=472f0c0a1&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdinceutics-essential-purifier-150-ml?_pos=1&amp;_sid=85546c272&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdinceutics-essential-scrub-100-g?_pos=1&amp;_sid=aee61eb38&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/search?options%5Bunavailable_products%5D=last&amp;options%5Bprefix%5D=last&amp;options%5Bfields%5D=title%2Cvendor%2Cproduct_type%2Cvariants.title&amp;q=ISDINCEUTICS+RETINAL+EYES+20ML</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdinceutics-salicylic-renewal-serum30ml?_pos=1&amp;_sid=67f169499&amp;_ss=r</t>
+  </si>
+  <si>
+    <t>Falabella</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72971956/Hidratante-facial-Isdin-Para-Piel-Normal-50-/72971956</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682163/Hidratante-Corporal-Ureadin-Utra-10-Isdin-para-Piel-seca-400-ml/12682163</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682128/Bloqueador-Solar-Eryfotona-AK-NMSC-Isdin-para-Piel-Sensible-50-ml/12682128</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682132/Bloqueador-Solar-Fusion-Water-con-Color-Isdin-para-Piel-Mixta-50-ml/12682132</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/29086847/Bloqueador-Solar-Foto-Ultra-100-Active-Unify-Isdin-para-Todo-tipo-de-piel-50-ml/29086847</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/29086848/Bloqueador-Solar-Fotoultra-Active-Unify-Color-50-ml-Isdin-para-Todo-tipo-de-piel-50-ml/29086848</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73148089/Protector-solar-FUSION-WATER-MAGIC-REPAIR-SPF50-50ML-Crema-ISDIN-Crema-50ml/73148089</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com/falabella-cl/product/80004010/Fotoprotector-Fusion-Water-Magic-Pediatrics-Spf-50-50Ml-Isdin/80004010</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/31652096/Serum-Isdinceutics-Rejuvenate-Flavo-C-Isdin-para-Todo-tipo-de-piel-30-ml/31652096</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/29073409/Tratamiento-Antiedad-Anti-arrugas-para-Rostro-Age-Reverse-Day-Isdin-50-ml/29073409</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682179/Contorno-de-Ojos-K-Ox-Eyes-Isdin-para-Piel-Normal-15-ml/12682179</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682154/Hidratante-Facial-Nutradeica-DS-Isdin-para-Piel-Grasa-50-ml/12682154</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73133689/Bloqueador-Fp-Invisible-Stick-Spf50-10G-en-barra-Isdin-10-gr/73133689</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682170/Tratamiento-antiedad-Age-Reverse-Night-Noche-Isdin-para-Piel-Normal-50-ml/12682170</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73259531/Protector-solar-Fotoprotector-Fusion-Water-Magic-By-Alcaraz-Emulsion-Isdin-50-ml/73259531</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/20233919/Hidratante-Facial-Isdinceutics-Hyaluronic-Concentrate-Isdin-para-Todo-tipo-de-piel-30-ml/20233919</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/19508501/Contorno-de-Ojos-Rejuvenate-Vital-Eyes-Noche-Isdin-para-Todo-tipo-de-piel-15-ml/19508501</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73051045/Protector-solar-Isdin-FotoUltra-100-Fotoprotecto-Spot-Prevent-Color-SPF-50+-Crema-ISDIN-Crema-50ml/73051045</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73148088/Protector-solar-Fusion-Water-MAgic-REPAIR-COLOR-SPF50-50ML-Crema-ISDIN-Crema-50ml/73148088</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73265847/Fotoprotector-ISDIN-Fusion-Gel-SPORT-SPF50-Protector-solar-corporal-para-el-deporte-Isdin-para-Todo-tipo-de-piel-100-ml/73265847</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73129676/Bloqueador-FP-GEL-CREAM-SPF50-250ML-Crema-ISDIN-Gel-250ml/73129676</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/37776295/Bloqueador-Solar-Fusion-Water-Color-Light-Isdin-para-Todo-tipo-de-piel-50-ml/37776295</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/46172384/Limpiador-Essential-Cleansing-Isdin-para-Todo-tipo-de-piel-200-ml/46172384</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/63668172/Bloqueador-Corporal-Adultos-Wet-Skin-Transparent-en-Spray-Isdin-250-ml/63668172</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/63668173/Tratamiento-antiedad-Noche-Isdinceutics-Retinal-Intense-Isdin-para-Todo-tipo-de-piel-50-ml/63668173</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72757444/Bloqueador-Liquido-Fusion-Water-Magic-SPF50-ISDIN-50-ml/72757444</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72914712/Locion-Babynaturals-Body-Lotion-Isdin-para-Bebes400-ml/72914712</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72914713/Jabon-Babynaturals-Gel-Shampoo-Isdin-para-Bebes-400-ml/72914713</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72914711/Crema-Babynaturals-Pomada-Isdin-para-Bebes-100-ml/72914711</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73233722/Suero-MELACLEAR-ADVANCED-SERUM-DESPIGMANTANTE-Isdin-para-Todo-tipo-de-piel-30-ml/73233722</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73390088/Protector-solar-Fotoprotector-Pediatrics-Stick-en-Barra-Isdin-20-Gr/73390088</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/122877665/Fotoprotector-Isdin-Uv-Mineral-Brush-Polvo-50spf-X-2g/122877666</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/122787136/Polvo-Compacto-Isdin-Fotoprotector-Spf50-Arena-10g/122787137</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/37776294/Bloqueador-Solar-Fusion-Water-Color-Bronze-Isdin-para-Todo-tipo-de-piel-50-ml/37776294</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682133/Bloqueador-Solar-Fusion-Water-Urban-Isdin-para-Piel-Mixta-50-ml/12682133</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73390092/Protector-solar-Fotoprotector-Fusion-Water-Magic-Glow-en-Crema-Isdin-50-ml/73390092</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/122877557/Fotoprotector-Isdin-Hydrolotion-+-50spf-200ml/122877558</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/123173276/Fotoprotector-Isdin-Hydro-Oil-SPF-30-Proteccion-Alta-X-200-Ml/123173278</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73531835/bloqueador-fp-fw-body-glow-spf-30-en-crema-isdin-200-ml/73531835</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/search?Ntt=FU+SPOT+PREVENT+SPF50+50ML</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73051046/Fotoprotector-para-labios-FP-LIPSTICK-SPF-50+-4G-Barra-ISDIN-4-g/73051046</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682168/Limpiador-Germisdin-Gel-de-Bano-Isdin-para-Piel-Normal-500-ml/12682168</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/125963015/locion-isdin-lambdapil-anticaida-x-125ml/125963016</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682156/Hidratante-Facial-Nutratopic-Pro-AMP-Emoliente-Isdin-para-Todo-tipo-de-piel-50-ml/12682156</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682157/Limpiador-Nutratopic-de-Bano-Isdin-para-Piel-Sensible-400-ml/12682157</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682158/Hidratante-Corporal-Nutratopic-Pro-AMP-Isdin-para-Piel-Sensible-400-ml/12682158</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/prod13940005/Tratamiento-Labios-Reparador-Stick-Isdin-4-Gr/73390089</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/prod13940005/Tratamiento-Labios-Reparador-Stick-Isdin-4-Gr/73390090</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/prod13940005/Tratamiento-Labios-Reparador-Stick-Isdin-4-Gr/73390091</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682153/Protector-para-Labios-Isdin-para-Todo-tipo-de-piel-4-g/12682153</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72970532/Balsamo-Reparador-Labial-Isdin-para-Todo-tipo-de-piel-30-ml/72970532</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682150/Tratamiento-para-Unas-Si-Nails-Isdin-para-Todo-tipo-de-piel-2.5-ml/12682150</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682151/Agua-Micelar-Solution-4-en-1-Isdin-para-Piel-Normal-400-ml/12682151</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682152/Agua-Micelar-Solution-4-en-1-Isdin-para-Piel-Normal-100-ml/12682152</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682160/Tratamiento-para-Pies-Ureadin-Podos-Isdin-para-Piel-Normal-75-ml/12682160</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/12682161/Tratamiento-para-Manos-Ureadin-Plus-Repair-Isdin-para-Piel-Normal-50-ml/12682161</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/46172382/Reafirmante-para-Cuerpo-Isdin-250-ml/46172382</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/73398122/Contorno-de-ojos-Ceutics-Hyaluronic-Eyes-Isdin-para-Todo-tipo-de-piel-15-gr/73398122</t>
+  </si>
+  <si>
+    <t>https://www.falabella.com.co/falabella-co/product/72971958/Hidratante-facial-Isdin-Para-Piel-Mixta-50-/72971958</t>
+  </si>
+  <si>
+    <t>Pasteur</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-eryfotona-ak-nmsc-fluido-spf-99-caja-50-ml-867250/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdin-eryfotona-night-emulsion-frasco-50-ml-867039/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-invisible-stick-fotoprotector-spf-50-frasco-10-g-867036/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-infantiles-isdin-pediatrics-stick-fotoprotector-barra-20-g-867041/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-maquillaje-dermoprotector-isdin-uv-mineral-brush-spf-50--tubo-2-g-867293/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fusion-fluido-spf-50--caja-50-ml-045228/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fotop--fusion-mineral-fluido-frasco-50-ml-867263/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fotoprotector-fusion-water-magic-by-alcaraz-frasco-50-ml-867038/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fusion-water-magic-fotoprotector-spf-50-frasco-50-ml-867015/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-fusion-water-magic-spf-50-color-medium-frasco-50-ml-867001/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-fusion-water-magic-spf-50-color-bronze-caja-50-ml-867003/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-fusion-water-magic-spf-50-color-light-frasco-50-ml-867002/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fusion-water-magic-urban-spf-30-frasco-50-ml-867268/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fotoprotector-fusion-water-magic-glow-frasco-50-ml-867045/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-infantiles-isdin-fusion-water-magic-spf-50-pediatric-frasco-50-ml-867215/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-isdin-fotoprotector-gel-crema-spf-50--tubo-250-ml-045222/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-infantiles-isdin-pediatrics-gel-crema-fotoprotector-spf-50-tubo-250-ml-867014/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-fotoprotec-isdin-hydro-lotion-spf-50-frasco-200-ml-867269/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-fotoprotector-hydrooil-spf-30-200-ml-867285/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-isdin-fotoprotector-fusion-gel-sport-spf-50-frasco-100-ml-867037/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-isdin-fotoprotector-transparen-spray-wet-skin-spf-50-frasco-250-ml-867009/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-corporales-isdin-fotoprotector-body-glow-spf-30-tubo-200-ml-867048/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fotoultra-redness-spf-50-frasco-50-ml-867032/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-isdin-fotoultra-100-fluido-spf-50--active-unify-caja-50-ml-867282/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-fotoultra-100-color-spf-50--active-unify-caja-50-ml-867287/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-fotoultra-100-spot-prevent-fluido-caja-50-ml-867281/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-foto-ultra-100-spot-prev-spf-50--color-frasco-50-ml-867027/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-faciales-fotoultra-age-repair-water-spf-50-caja-50-ml-867254/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-maquillaje-dermoprotector-con-color-isdin-fotoprotector-fusion-water-magic-repair-color-frasco-50-ml-867035/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-protector-labial-spf-50-barra-4-g-867259/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-protector-labial-hv-spf-30-barra-4-g-867260/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-protector-labial-spf-30-barra-4-g-867261/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-otros-tratamientos-shampoo-y-acondicionador-isdin-dayl-shampoo-ultra-suave-frasco-400-ml-867271/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-jabones-y-limpiadores-germisdin-gel-bano-frasco-500-ml-867265/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-protector-cutaneo-isdin-cicapost-crema-tubo-50-g-867047/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-otros-tratamientos-anticaida-isdin-lambdapil-champu-anticaida-frasco-200-ml-867272/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-otros-tratamientos-anticaida-isdin-lambdapil-locion-anticaida-melatonin-spray-100-ml-867046/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdin-nutradeica-ds-gel-crema-caja-50-ml-867255/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-otros-tratamientos-anticaspa-isdin-nutradeica-champu-anticaspa-grasa-frasco-200-ml-867273/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-nutratopic-pro-amp-piel-react-crema-caja-50-ml-867310/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-jabones-y-limpiadores-nutratopic-pro-amp-gel-bano-frasco-400-ml-867312/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-nutratopic-pro-amp-emoliente-locion-frasco-400-ml-867311/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-proteccion-solar-hidratantes-isdin-baby-naturals-nutraisdin-pomada-del-panal-tubo-100-ml-867020/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-proteccion-solar-hidratantes-isdin-babynaturals-body-lotion-frasco-400-ml-867021/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-proteccion-solar-bano-isdin-baby-naturals-nutraisdin-gel-champu-frasco-400-ml-867019/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-labial-rojo-barra-4-g-867043/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-labial-rosa-barra-4-g-867044/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-labial-granate-barra-4-g-867042/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-labial-barra-4-g-867262/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-labial-fluido-tubo-10-ml-867010/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-cuidado-de-labios-isdin-reparador-balsamo-labial-10-ml-867022/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-otros-tratamientos-ciudado-de-las-unas-isdin-si-nails-caja-2-5-ml-867264/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-medicamentos-y-tratamientos--niogermox-solucion-topica-8--caja-3-3-ml-867253/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-limpiadores-y-desmaquillantes-isdin-micellar-solution-frasco-400-ml-867251/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-limpiadores-y-desmaquillantes-isdin-micellar-solution-frasco-100-ml-867256/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-jabones-y-limpiadores-ureadin-bath-gel-frasco-400-ml-867401/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-podos-pies-secos-caja-75-ml-045819/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-ultra-10-locion-caja-200-ml-867212/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-ultra-10-locion-caja-400-ml-867213/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-isdin-ureadin-lotion-10-frasco-1000-ml-867011/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-ultra-20-crema-caja-100-ml-867214/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-ultra-30-exfoliante-crema-caja-50-ml-045827/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-ureadin-manos-plus-repair-crema-tubo-50-ml-867267/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-reductores-y-reafirmantes-isdin-woman-crema-reafirmante-tubo-200-ml-867005/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-hidratantes-isdin-woman-crema-anti-estrias-tubo-250-ml-867004/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-reductores-y-reafirmantes-cuidado-intimo-isdin-woman-higiene-intima-gel-frasco-200-ml-867028/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-mascarillas-y-serum-isdinceutics-flavo-c-serum-caja-30-ml-867258/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-contorno-de-ojos-isdinceutics-k-ox-eyes-crema-caja-15-g-867257/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-contorno-de-ojos-isdinceutics-vital-eyes-caja-15-g-867280/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-contorno-de-ojos-isdinceutics-hyaluronic-eyes-gel-pote-15-g-867040/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-mascarillas-y-serum-isdin-hyaluronic-concentrate-serum-frasco-30-ml-867276/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdinceutics-hyaluronic-moisture-normal-to-dry-skin-caja-50-g-867025/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdinceutics-hyaluronic-moisture-normal-to-dry-skin-refill-caja-50-g-867026/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdinceutics-hyaluronic-moisture-oily---combination-skin-caja-50-g-867023/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-hidratantes-isdinceutics-hyaluronic-moisture-oily---combination-skin-refill-caja-50-g-867024/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-limpiadores-y-desmaquillantes-isdinceutics-essential-cleansing-aceite-limpiador-frasco-200-ml-867008/p</t>
+  </si>
+  <si>
+    <t>https://www.farmaciaspasteur.com.co/dermocosmetica-mascarillas-y-serum-mascarillas-y-serum-isdinceutics-retinal-intense-serum-facial-frasco-50-ml-867029/p</t>
   </si>
 </sst>
 </file>
@@ -2473,13 +3091,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C4ECE9E-4A28-6340-B936-CE442F4057E5}">
-  <dimension ref="A1:N514"/>
+  <dimension ref="A1:N718"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="62.33203125" customWidth="1"/>
     <col min="2" max="2" width="29.5" customWidth="1"/>
     <col min="3" max="3" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
+    <col min="4" max="4" width="255.58203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
@@ -10255,9 +10873,2871 @@
         <v>632</v>
       </c>
     </row>
+    <row r="515" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A515" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B515" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C515" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D515" s="3" t="s">
+        <v>634</v>
+      </c>
+    </row>
+    <row r="516" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A516" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B516" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C516" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D516" s="5" t="s">
+        <v>635</v>
+      </c>
+    </row>
+    <row r="517" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A517" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B517" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C517" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D517" s="5" t="s">
+        <v>636</v>
+      </c>
+    </row>
+    <row r="518" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A518" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B518" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="C518" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D518" s="5" t="s">
+        <v>637</v>
+      </c>
+    </row>
+    <row r="519" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A519" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B519" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C519" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D519" s="5" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="520" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A520" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B520" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C520" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D520" s="5" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="521" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A521" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B521" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C521" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D521" s="5" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="522" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A522" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B522" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C522" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D522" s="5" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="523" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A523" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B523" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C523" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D523" s="5" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="524" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A524" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B524" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C524" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D524" s="5" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="525" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A525" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B525" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C525" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D525" s="5" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="526" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A526" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B526" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C526" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D526" s="5" t="s">
+        <v>645</v>
+      </c>
+    </row>
+    <row r="527" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A527" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B527" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C527" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D527" s="5" t="s">
+        <v>646</v>
+      </c>
+    </row>
+    <row r="528" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A528" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B528" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C528" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D528" s="5" t="s">
+        <v>647</v>
+      </c>
+    </row>
+    <row r="529" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A529" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B529" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C529" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D529" s="3" t="s">
+        <v>648</v>
+      </c>
+    </row>
+    <row r="530" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A530" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B530" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C530" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D530" s="5" t="s">
+        <v>649</v>
+      </c>
+    </row>
+    <row r="531" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A531" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B531" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C531" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D531" s="5" t="s">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="532" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A532" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B532" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C532" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D532" s="5" t="s">
+        <v>651</v>
+      </c>
+    </row>
+    <row r="533" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A533" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B533" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C533" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D533" s="5" t="s">
+        <v>652</v>
+      </c>
+    </row>
+    <row r="534" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A534" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B534" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C534" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D534" s="5" t="s">
+        <v>653</v>
+      </c>
+    </row>
+    <row r="535" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A535" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B535" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C535" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D535" s="5" t="s">
+        <v>654</v>
+      </c>
+    </row>
+    <row r="536" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A536" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B536" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C536" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D536" s="5" t="s">
+        <v>655</v>
+      </c>
+    </row>
+    <row r="537" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A537" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B537" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C537" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D537" s="5" t="s">
+        <v>656</v>
+      </c>
+    </row>
+    <row r="538" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A538" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B538" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C538" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D538" s="5" t="s">
+        <v>657</v>
+      </c>
+    </row>
+    <row r="539" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A539" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B539" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C539" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D539" s="3" t="s">
+        <v>658</v>
+      </c>
+    </row>
+    <row r="540" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A540" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B540" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C540" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D540" s="3" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="541" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A541" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="B541" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C541" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D541" s="3" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="542" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A542" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B542" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C542" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D542" s="3" t="s">
+        <v>661</v>
+      </c>
+    </row>
+    <row r="543" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A543" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B543" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C543" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D543" s="3" t="s">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="544" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A544" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B544" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C544" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D544" s="3" t="s">
+        <v>663</v>
+      </c>
+    </row>
+    <row r="545" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A545" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B545" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C545" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D545" s="3" t="s">
+        <v>664</v>
+      </c>
+    </row>
+    <row r="546" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A546" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B546" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C546" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D546" s="3" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="547" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A547" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B547" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C547" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D547" s="3" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="548" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A548" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B548" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C548" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D548" s="3" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="549" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A549" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B549" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C549" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D549" s="3" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="550" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A550" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B550" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C550" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D550" s="3" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="551" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A551" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B551" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C551" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D551" s="3" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="552" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A552" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B552" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C552" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D552" s="3" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="553" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A553" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B553" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C553" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D553" s="3" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="554" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A554" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B554" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C554" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D554" s="3" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="555" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A555" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B555" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C555" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D555" s="3" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="556" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A556" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B556" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C556" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D556" s="3" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="557" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A557" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B557" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C557" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D557" s="3" t="s">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="558" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A558" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B558" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C558" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D558" s="3" t="s">
+        <v>677</v>
+      </c>
+    </row>
+    <row r="559" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A559" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B559" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C559" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D559" s="3" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="560" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A560" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B560" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C560" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D560" s="3" t="s">
+        <v>679</v>
+      </c>
+    </row>
+    <row r="561" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A561" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B561" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C561" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D561" s="3" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="562" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A562" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B562" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C562" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D562" s="3" t="s">
+        <v>681</v>
+      </c>
+    </row>
+    <row r="563" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A563" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B563" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C563" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D563" s="3" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="564" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A564" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B564" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C564" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D564" s="3" t="s">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="565" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A565" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B565" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C565" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D565" s="3" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="566" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A566" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B566" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C566" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D566" s="3" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="567" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A567" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B567" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C567" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D567" s="3" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="568" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A568" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B568" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C568" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D568" s="3" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="569" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A569" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B569" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C569" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D569" s="3" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="570" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A570" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B570" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C570" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D570" s="3" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="571" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A571" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B571" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C571" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D571" s="3" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="572" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A572" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B572" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C572" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D572" s="3" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="573" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A573" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B573" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C573" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D573" s="3" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="574" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A574" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B574" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C574" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D574" s="3" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="575" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A575" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B575" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C575" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D575" s="3" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="576" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A576" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B576" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C576" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D576" s="3" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="577" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A577" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="B577" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C577" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D577" s="3" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="578" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A578" s="3" t="s">
+        <v>344</v>
+      </c>
+      <c r="B578" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C578" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D578" s="3" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="579" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A579" s="3" t="s">
+        <v>346</v>
+      </c>
+      <c r="B579" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C579" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D579" s="3" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="580" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A580" s="3" t="s">
+        <v>348</v>
+      </c>
+      <c r="B580" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C580" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D580" s="3" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="581" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A581" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="B581" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C581" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="D581" s="3" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="582" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A582" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B582" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C582" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D582" s="5" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="583" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A583" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B583" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C583" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D583" s="3" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="584" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A584" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B584" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C584" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D584" s="3" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="585" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A585" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B585" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C585" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D585" s="5" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="586" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A586" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B586" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C586" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D586" s="5" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="587" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A587" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B587" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C587" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D587" s="5" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="588" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A588" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B588" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C588" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D588" s="5" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="589" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A589" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B589" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C589" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D589" s="5" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="590" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A590" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B590" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C590" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D590" s="5" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="591" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A591" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B591" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C591" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D591" s="5" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="592" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A592" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B592" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C592" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D592" s="5" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="593" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A593" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B593" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C593" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D593" s="3" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="594" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A594" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B594" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C594" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D594" s="5" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="595" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A595" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B595" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C595" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D595" s="5" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="596" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A596" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B596" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C596" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D596" s="5" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="597" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A597" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B597" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C597" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D597" s="5" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="598" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A598" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B598" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C598" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D598" s="5" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="599" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A599" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B599" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C599" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D599" s="5" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="600" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A600" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B600" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C600" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D600" s="5" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="601" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A601" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B601" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C601" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D601" s="5" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="602" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A602" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B602" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C602" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D602" s="5" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="603" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A603" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B603" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C603" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D603" s="5" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="604" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A604" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B604" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C604" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D604" s="5" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="605" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A605" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B605" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C605" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D605" s="5" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="606" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A606" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B606" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C606" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D606" s="5" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="607" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A607" s="28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B607" s="29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C607" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D607" s="29" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="608" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A608" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B608" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C608" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D608" s="5" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="609" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A609" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B609" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C609" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D609" s="3" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="610" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A610" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B610" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C610" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D610" s="3" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="611" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A611" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B611" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C611" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D611" s="5" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="612" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A612" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B612" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C612" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D612" s="3" t="s">
+        <v>732</v>
+      </c>
+    </row>
+    <row r="613" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A613" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B613" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C613" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D613" s="3" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="614" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A614" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="B614" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C614" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D614" s="3" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="615" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A615" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B615" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C615" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D615" s="3" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="616" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A616" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B616" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C616" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D616" s="3" t="s">
+        <v>736</v>
+      </c>
+    </row>
+    <row r="617" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A617" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B617" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C617" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D617" s="3" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="618" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A618" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B618" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C618" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D618" s="3" t="s">
+        <v>738</v>
+      </c>
+    </row>
+    <row r="619" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A619" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B619" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C619" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D619" s="3" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="620" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A620" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B620" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C620" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D620" s="3" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="621" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A621" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B621" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C621" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D621" s="3" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="622" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A622" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B622" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C622" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D622" s="3" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="623" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A623" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="B623" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C623" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D623" s="3" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="624" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A624" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B624" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C624" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D624" s="3" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="625" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A625" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B625" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C625" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="D625" s="3" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="626" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A626" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B626" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C626" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D626" s="5" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="627" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A627" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B627" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C627" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D627" s="5" t="s">
+        <v>746</v>
+      </c>
+    </row>
+    <row r="628" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A628" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B628" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C628" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D628" s="5" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="629" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A629" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B629" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C629" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D629" s="5" t="s">
+        <v>748</v>
+      </c>
+    </row>
+    <row r="630" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A630" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B630" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C630" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D630" s="5" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="631" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A631" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B631" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C631" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D631" s="5" t="s">
+        <v>750</v>
+      </c>
+    </row>
+    <row r="632" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A632" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B632" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C632" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D632" s="5" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="633" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A633" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B633" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C633" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D633" s="5" t="s">
+        <v>752</v>
+      </c>
+    </row>
+    <row r="634" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A634" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B634" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C634" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D634" s="5" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="635" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A635" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B635" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C635" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D635" s="5" t="s">
+        <v>754</v>
+      </c>
+    </row>
+    <row r="636" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A636" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B636" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C636" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D636" s="5" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="637" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A637" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B637" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C637" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D637" s="5" t="s">
+        <v>756</v>
+      </c>
+    </row>
+    <row r="638" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A638" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B638" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C638" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D638" s="3" t="s">
+        <v>757</v>
+      </c>
+      <c r="E638" s="3"/>
+      <c r="F638" s="5"/>
+      <c r="G638" s="3"/>
+    </row>
+    <row r="639" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A639" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B639" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C639" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D639" s="5" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="640" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A640" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B640" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C640" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D640" s="5" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="641" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A641" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B641" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C641" s="3" t="s">
+        <v>701</v>
+      </c>
+      <c r="D641" s="5" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="642" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A642" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B642" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C642" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D642" s="5" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="643" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A643" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B643" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C643" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D643" s="5" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="644" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A644" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B644" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C644" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D644" s="5" t="s">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="645" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A645" s="3" t="s">
+        <v>234</v>
+      </c>
+      <c r="B645" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C645" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D645" s="5" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="646" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A646" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="B646" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C646" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D646" s="5" t="s">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="647" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A647" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B647" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C647" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D647" s="5" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="648" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A648" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B648" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C648" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D648" s="5" t="s">
+        <v>768</v>
+      </c>
+    </row>
+    <row r="649" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A649" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B649" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C649" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D649" s="5" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="650" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A650" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B650" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C650" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D650" s="5" t="s">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="651" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A651" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B651" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C651" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D651" s="5" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="652" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A652" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="B652" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C652" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D652" s="5" t="s">
+        <v>772</v>
+      </c>
+    </row>
+    <row r="653" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A653" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B653" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C653" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D653" s="5" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="654" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A654" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="B654" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C654" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D654" s="5" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="655" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A655" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="B655" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C655" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D655" s="5" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="656" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A656" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B656" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C656" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D656" s="5" t="s">
+        <v>776</v>
+      </c>
+    </row>
+    <row r="657" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A657" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B657" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C657" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D657" s="5" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="658" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A658" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B658" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C658" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D658" s="5" t="s">
+        <v>778</v>
+      </c>
+    </row>
+    <row r="659" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A659" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B659" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C659" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D659" s="5" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="660" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A660" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="B660" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C660" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D660" s="5" t="s">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="661" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A661" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B661" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C661" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D661" s="5" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="662" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A662" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B662" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C662" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D662" s="5" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="663" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A663" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B663" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C663" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D663" s="5" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="664" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A664" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="B664" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C664" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D664" s="5" t="s">
+        <v>784</v>
+      </c>
+    </row>
+    <row r="665" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A665" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B665" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C665" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D665" s="5" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="666" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A666" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B666" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C666" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D666" s="5" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="667" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A667" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B667" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C667" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D667" s="5" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="668" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A668" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B668" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C668" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D668" s="5" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="669" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A669" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B669" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C669" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D669" s="5" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="670" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A670" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B670" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C670" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D670" s="5" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="671" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A671" s="3" t="s">
+        <v>371</v>
+      </c>
+      <c r="B671" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C671" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D671" s="5" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="672" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A672" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B672" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C672" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D672" s="5" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="673" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A673" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B673" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C673" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D673" s="5" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="674" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A674" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="B674" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C674" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D674" s="5" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="675" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A675" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B675" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C675" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D675" s="5" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="676" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A676" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B676" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C676" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D676" s="5" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="677" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A677" s="3" t="s">
+        <v>278</v>
+      </c>
+      <c r="B677" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C677" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D677" s="5" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="678" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A678" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="B678" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C678" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D678" s="5" t="s">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="679" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A679" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B679" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C679" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D679" s="5" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="680" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A680" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B680" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C680" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D680" s="5" t="s">
+        <v>800</v>
+      </c>
+    </row>
+    <row r="681" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A681" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B681" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C681" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D681" s="5" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="682" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A682" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="B682" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C682" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D682" s="5" t="s">
+        <v>802</v>
+      </c>
+    </row>
+    <row r="683" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A683" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="B683" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C683" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D683" s="5" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="684" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A684" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B684" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C684" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D684" s="5" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="685" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A685" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B685" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C685" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D685" s="5" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="686" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A686" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B686" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C686" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D686" s="5" t="s">
+        <v>806</v>
+      </c>
+    </row>
+    <row r="687" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A687" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B687" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C687" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D687" s="5" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="688" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A688" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B688" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C688" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D688" s="5" t="s">
+        <v>808</v>
+      </c>
+    </row>
+    <row r="689" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A689" s="3" t="s">
+        <v>385</v>
+      </c>
+      <c r="B689" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C689" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D689" s="5" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="690" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A690" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B690" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C690" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D690" s="5" t="s">
+        <v>810</v>
+      </c>
+    </row>
+    <row r="691" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A691" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B691" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C691" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D691" s="5" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="692" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A692" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B692" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C692" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D692" s="5" t="s">
+        <v>812</v>
+      </c>
+    </row>
+    <row r="693" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A693" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B693" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C693" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D693" s="5" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="694" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A694" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B694" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C694" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D694" s="5" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="695" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A695" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B695" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C695" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D695" s="5" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="696" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A696" s="3" t="s">
+        <v>390</v>
+      </c>
+      <c r="B696" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C696" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D696" s="5" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="697" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A697" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B697" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C697" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D697" s="5" t="s">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="698" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A698" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="B698" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C698" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D698" s="5" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="699" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A699" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B699" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C699" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D699" s="5" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="700" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A700" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B700" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C700" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D700" s="5" t="s">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="701" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A701" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B701" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C701" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D701" s="5" t="s">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="702" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A702" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B702" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C702" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D702" s="5" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="703" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A703" s="3" t="s">
+        <v>312</v>
+      </c>
+      <c r="B703" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C703" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D703" s="5" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="704" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A704" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="B704" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C704" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D704" s="5" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="705" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A705" s="3" t="s">
+        <v>318</v>
+      </c>
+      <c r="B705" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C705" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D705" s="5" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="706" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A706" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B706" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C706" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D706" s="5" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="707" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A707" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="B707" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C707" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D707" s="5" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="708" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A708" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B708" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C708" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D708" s="5" t="s">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="709" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A709" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B709" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C709" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D709" s="5" t="s">
+        <v>829</v>
+      </c>
+    </row>
+    <row r="710" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A710" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B710" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C710" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D710" s="5" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="711" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A711" s="3" t="s">
+        <v>330</v>
+      </c>
+      <c r="B711" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C711" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D711" s="5" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="712" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A712" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B712" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C712" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D712" s="5" t="s">
+        <v>832</v>
+      </c>
+    </row>
+    <row r="713" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A713" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B713" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C713" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D713" s="5" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="714" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A714" s="3" t="s">
+        <v>332</v>
+      </c>
+      <c r="B714" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C714" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D714" s="5" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="715" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A715" s="3" t="s">
+        <v>334</v>
+      </c>
+      <c r="B715" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C715" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D715" s="5" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="716" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A716" s="3" t="s">
+        <v>336</v>
+      </c>
+      <c r="B716" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C716" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D716" s="5" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="717" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A717" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B717" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C717" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D717" s="5" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="718" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A718" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B718" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C718" s="3" t="s">
+        <v>761</v>
+      </c>
+      <c r="D718" s="5" t="s">
+        <v>838</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D514" xr:uid="{2C4ECE9E-4A28-6340-B936-CE442F4057E5}"/>
+  <autoFilter ref="A1:D581" xr:uid="{2C4ECE9E-4A28-6340-B936-CE442F4057E5}"/>
   <phoneticPr fontId="4" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D704" r:id="rId1" xr:uid="{C4A764D9-65E4-467B-BC7B-5C3E51C52CDA}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Ajuste código LASKIN e inclusión de Coverage al seguimiento de laskin
</commit_message>
<xml_diff>
--- a/data/productos.xlsx
+++ b/data/productos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AMSIERRA\Documents\ISDIN_Shopping_de_precios\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27B9B3C0-7256-407C-9BFB-D7E5E4C512BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7EFF4E1-9A64-4EAD-AF65-0D75E7F3D9BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{60233B49-B589-B346-B71C-4D486694C55A}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$676</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$D$682</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2704" uniqueCount="787">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2728" uniqueCount="793">
   <si>
     <t>Producto</t>
   </si>
@@ -2400,6 +2400,24 @@
   </si>
   <si>
     <t>https://lineaestetica.co/product/isdin-instant-flash-efecto-lifting/?attribute_pa_unidades=1-ampolla</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-coverage-1-0-pearl?_pos=2&amp;_psq=COVERAGE&amp;_ss=e&amp;_v=1.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-coverage-2-0-beige?_pos=1&amp;_psq=COVERAGE&amp;_ss=e&amp;_v=2.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/cicapost-crema-50-gr-isdin?_pos=2&amp;_psq=cica&amp;_ss=e&amp;_v=1.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-coverage-3-0-sand?_pos=1&amp;_psq=COVERAGE&amp;_ss=e&amp;_v=1.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-coverage-4-0-golden?_pos=1&amp;_psq=COVERAGE&amp;_ss=e&amp;_v=3.0</t>
+  </si>
+  <si>
+    <t>https://laskin.com.co/products/isdin-coverage-5-0-bronze?_pos=1&amp;_psq=COVERAGE&amp;_ss=e&amp;_v=3.0</t>
   </si>
 </sst>
 </file>
@@ -2578,7 +2596,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2628,6 +2646,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="15" fontId="6" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -2958,7 +2979,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C4ECE9E-4A28-6340-B936-CE442F4057E5}">
-  <dimension ref="A1:M676"/>
+  <dimension ref="A1:M682"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="62.3984375" customWidth="1"/>
@@ -12952,7 +12973,92 @@
         <v>763</v>
       </c>
     </row>
+    <row r="677" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A677" s="3" t="s">
+        <v>734</v>
+      </c>
+      <c r="B677" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C677" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D677" s="41" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="678" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A678" s="3" t="s">
+        <v>735</v>
+      </c>
+      <c r="B678" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C678" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D678" s="41" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="679" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A679" s="3" t="s">
+        <v>736</v>
+      </c>
+      <c r="B679" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C679" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D679" s="43" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="680" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A680" s="3" t="s">
+        <v>737</v>
+      </c>
+      <c r="B680" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C680" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D680" s="43" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="681" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A681" s="3" t="s">
+        <v>738</v>
+      </c>
+      <c r="B681" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C681" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D681" s="43" t="s">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="682" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A682" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B682" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C682" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="D682" s="41" t="s">
+        <v>789</v>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D682" xr:uid="{2C4ECE9E-4A28-6340-B936-CE442F4057E5}"/>
   <phoneticPr fontId="4" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="D638" r:id="rId1" xr:uid="{C4A764D9-65E4-467B-BC7B-5C3E51C52CDA}"/>
@@ -13019,8 +13125,11 @@
     <hyperlink ref="D126" r:id="rId62" xr:uid="{B798115A-2494-40DA-9647-3F9D20A7DD75}"/>
     <hyperlink ref="D131" r:id="rId63" xr:uid="{C601D573-7598-460B-96F9-1A1FA18576D2}"/>
     <hyperlink ref="D132" r:id="rId64" xr:uid="{15EA25BC-1188-4E7B-9977-31DE4FE4EE9A}"/>
+    <hyperlink ref="D679" r:id="rId65" xr:uid="{96BA4FB7-0FCC-4C86-BE00-F7E6F4184E7D}"/>
+    <hyperlink ref="D680" r:id="rId66" xr:uid="{FC45698F-DD69-42C9-B450-C81797AA090B}"/>
+    <hyperlink ref="D681" r:id="rId67" xr:uid="{61D7CAA3-790C-47E0-9A37-6C45A4481FA1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId65"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId68"/>
 </worksheet>
 </file>
</xml_diff>